<commit_message>
Evento #2 registrado en reporte_2026-05-30.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-05-30.xlsx
+++ b/datos/excel/reporte_2026-05-30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,51 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>00:50:46</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>468.75</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-25.46</v>
+      </c>
+      <c r="G3" t="n">
+        <v>90.91</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>945.3 Hz | 1421.9 Hz | 1906.2 Hz</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2502</v>
+      </c>
+      <c r="J3" t="n">
+        <v>68</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>🚨 SÍ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evento #1 registrado en reporte_2026-05-30.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-05-30.xlsx
+++ b/datos/excel/reporte_2026-05-30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -560,6 +560,51 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>🚨 SÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>00:54:42</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>320.31</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-28.45</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>648.4 Hz | 937.5 Hz | 1234.4 Hz</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>2527</v>
+      </c>
+      <c r="J4" t="n">
+        <v>16521</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evento #3 registrado en reporte_2026-05-30.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-05-30.xlsx
+++ b/datos/excel/reporte_2026-05-30.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1238,6 +1238,51 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>01:31:51</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>468.75</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-20.49</v>
+      </c>
+      <c r="G19" t="n">
+        <v>98.67</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>945.3 Hz | 1421.9 Hz | 1906.2 Hz</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>2529</v>
+      </c>
+      <c r="J19" t="n">
+        <v>57</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>🚨 SÍ</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>